<commit_message>
feat: interactive organigram with React Flow, help page, and direct editing sidebar
</commit_message>
<xml_diff>
--- a/info/usuarios_superiores_organigrama_oficial.xlsx
+++ b/info/usuarios_superiores_organigrama_oficial.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tarantoms-my.sharepoint.com/personal/gautop_taranto_com_ar/Documents/Documentos/Material Soporte/03_Taranto/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tarantoms-my.sharepoint.com/personal/gautop_taranto_com_ar/Documents/Documentos/PROYECTOS APP/Organigrama/info/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_EB5568DFEFB1EA404877F79ABD761C678F691EAA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BB21CDDB-79C9-424C-A8E1-9FAB6AF10CBF}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="11_EB5568DFEFB1EA404877F79ABD761C678F691EAA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{677A9D51-16F5-4E90-B49F-ED0A716CCEF9}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1587,6 +1587,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:U81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1672,7 +1673,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>21</v>
       </c>
@@ -1737,7 +1738,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>21</v>
       </c>
@@ -1802,7 +1803,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>21</v>
       </c>
@@ -1867,7 +1868,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>21</v>
       </c>
@@ -1932,7 +1933,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>21</v>
       </c>
@@ -1997,7 +1998,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>21</v>
       </c>
@@ -2062,7 +2063,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>21</v>
       </c>
@@ -2127,7 +2128,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>21</v>
       </c>
@@ -2192,7 +2193,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>21</v>
       </c>
@@ -2255,7 +2256,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>21</v>
       </c>
@@ -2320,7 +2321,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>21</v>
       </c>
@@ -2383,7 +2384,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>21</v>
       </c>
@@ -2448,7 +2449,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>91</v>
       </c>
@@ -2511,7 +2512,7 @@
       </c>
       <c r="U14" s="2"/>
     </row>
-    <row r="15" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>91</v>
       </c>
@@ -2572,7 +2573,7 @@
       </c>
       <c r="U15" s="2"/>
     </row>
-    <row r="16" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>91</v>
       </c>
@@ -2637,7 +2638,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="17" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>91</v>
       </c>
@@ -2763,7 +2764,7 @@
       </c>
       <c r="U18" s="2"/>
     </row>
-    <row r="19" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>119</v>
       </c>
@@ -3001,7 +3002,7 @@
       </c>
       <c r="U22" s="2"/>
     </row>
-    <row r="23" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:21" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>150</v>
       </c>
@@ -3066,7 +3067,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="24" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:21" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>150</v>
       </c>
@@ -3125,7 +3126,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="25" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>150</v>
       </c>
@@ -3186,7 +3187,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="26" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>150</v>
       </c>
@@ -3245,7 +3246,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="27" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>150</v>
       </c>
@@ -3308,7 +3309,7 @@
       </c>
       <c r="U27" s="2"/>
     </row>
-    <row r="28" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>196</v>
       </c>
@@ -3371,7 +3372,7 @@
       </c>
       <c r="U28" s="2"/>
     </row>
-    <row r="29" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>196</v>
       </c>
@@ -3422,7 +3423,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="30" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:21" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>196</v>
       </c>
@@ -3473,7 +3474,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="31" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>196</v>
       </c>
@@ -3532,7 +3533,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="32" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>196</v>
       </c>
@@ -3591,7 +3592,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="33" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>196</v>
       </c>
@@ -3650,7 +3651,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="34" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>196</v>
       </c>
@@ -3713,7 +3714,7 @@
       </c>
       <c r="U34" s="2"/>
     </row>
-    <row r="35" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:21" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>196</v>
       </c>
@@ -3772,7 +3773,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="36" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:21" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>196</v>
       </c>
@@ -3837,7 +3838,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="37" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>196</v>
       </c>
@@ -3896,7 +3897,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="38" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>61</v>
       </c>
@@ -3947,7 +3948,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="39" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>61</v>
       </c>
@@ -4006,7 +4007,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="40" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>61</v>
       </c>
@@ -4057,7 +4058,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="41" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>61</v>
       </c>
@@ -4106,7 +4107,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="42" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:21" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>61</v>
       </c>
@@ -4169,7 +4170,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="43" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>61</v>
       </c>
@@ -4220,7 +4221,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="44" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>61</v>
       </c>
@@ -4271,7 +4272,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="45" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>61</v>
       </c>
@@ -4322,7 +4323,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="46" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>61</v>
       </c>
@@ -4373,7 +4374,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="47" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>61</v>
       </c>
@@ -4414,7 +4415,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="48" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:21" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>61</v>
       </c>
@@ -4465,7 +4466,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="49" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>61</v>
       </c>
@@ -4516,7 +4517,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="50" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:21" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>273</v>
       </c>
@@ -4581,7 +4582,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="51" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>195</v>
       </c>
@@ -4646,7 +4647,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="52" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>195</v>
       </c>
@@ -4709,7 +4710,7 @@
       </c>
       <c r="U52" s="2"/>
     </row>
-    <row r="53" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>195</v>
       </c>
@@ -4772,7 +4773,7 @@
       </c>
       <c r="U53" s="2"/>
     </row>
-    <row r="54" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>195</v>
       </c>
@@ -4835,7 +4836,7 @@
       </c>
       <c r="U54" s="2"/>
     </row>
-    <row r="55" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>195</v>
       </c>
@@ -4900,7 +4901,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="56" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:21" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>195</v>
       </c>
@@ -4961,7 +4962,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="57" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>195</v>
       </c>
@@ -5026,7 +5027,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="58" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>195</v>
       </c>
@@ -5089,7 +5090,7 @@
       </c>
       <c r="U58" s="2"/>
     </row>
-    <row r="59" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>109</v>
       </c>
@@ -5154,7 +5155,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="60" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>109</v>
       </c>
@@ -5217,7 +5218,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="61" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>109</v>
       </c>
@@ -5280,7 +5281,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="62" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>109</v>
       </c>
@@ -5343,7 +5344,7 @@
       </c>
       <c r="U62" s="2"/>
     </row>
-    <row r="63" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>109</v>
       </c>
@@ -5406,7 +5407,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="64" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>109</v>
       </c>
@@ -5471,7 +5472,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="65" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>109</v>
       </c>
@@ -5536,7 +5537,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="66" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>321</v>
       </c>
@@ -5601,7 +5602,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="67" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>321</v>
       </c>
@@ -5652,7 +5653,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="68" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>321</v>
       </c>
@@ -5703,7 +5704,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="69" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>73</v>
       </c>
@@ -5766,7 +5767,7 @@
       </c>
       <c r="U69" s="2"/>
     </row>
-    <row r="70" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>73</v>
       </c>
@@ -5829,7 +5830,7 @@
       </c>
       <c r="U70" s="2"/>
     </row>
-    <row r="71" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>73</v>
       </c>
@@ -5890,7 +5891,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="72" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>73</v>
       </c>
@@ -5955,7 +5956,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="73" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>73</v>
       </c>
@@ -6018,7 +6019,7 @@
       </c>
       <c r="U73" s="2"/>
     </row>
-    <row r="74" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>73</v>
       </c>
@@ -6069,7 +6070,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="75" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>73</v>
       </c>
@@ -6130,7 +6131,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="76" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>73</v>
       </c>
@@ -6193,7 +6194,7 @@
       </c>
       <c r="U76" s="2"/>
     </row>
-    <row r="77" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>73</v>
       </c>
@@ -6254,7 +6255,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="78" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>73</v>
       </c>
@@ -6315,7 +6316,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="79" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>365</v>
       </c>
@@ -6380,7 +6381,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="80" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>365</v>
       </c>
@@ -6431,7 +6432,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="81" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>365</v>
       </c>
@@ -6497,7 +6498,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U81" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:U81" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="7">
+      <filters>
+        <filter val="Caballero, Cecilia"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>